<commit_message>
progress: 61 village workbooks (sivaramans-llin 2026-10-10T15:40:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Panpakkam_13.376354_80.132208.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Panpakkam_13.376354_80.132208.xlsx
@@ -2090,6 +2090,11 @@
           <t>223</t>
         </is>
       </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 2A, 2B, 2C, 3, 4, 5, 6, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -2097,6 +2102,11 @@
           <t>224</t>
         </is>
       </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13A, 13B, 14A, 14B, 14C, 14D, 15, 16, 17A, 17B, 18A, 18B, 19, 1A, 1B, 2, 20, 21, 22, 23, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -2104,6 +2114,11 @@
           <t>225</t>
         </is>
       </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -2111,6 +2126,11 @@
           <t>226</t>
         </is>
       </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3A, 3B, 4A, 4B, 5A, 5B, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -2118,6 +2138,11 @@
           <t>227</t>
         </is>
       </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 1A, 1B, 2, 3A, 3B, 4A1, 4A2, 4B, 4B1, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -2125,6 +2150,11 @@
           <t>228</t>
         </is>
       </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 1A, 1B, 2A, 2B, 3, 4A, 4B, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -2132,6 +2162,11 @@
           <t>229</t>
         </is>
       </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3, 4, 5A, 5B, 6, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -2139,6 +2174,11 @@
           <t>23</t>
         </is>
       </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 42, 43, 44, 45, 46, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -2146,6 +2186,11 @@
           <t>230</t>
         </is>
       </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 1A, 1B, 2A, 2B, 3A, 3B, 4A, 4B, 5A, 5B, 6A, 6B, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -2153,6 +2198,11 @@
           <t>231</t>
         </is>
       </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>1, 10A1A, 10A2, 10B, 11A, 11B1A, 11B1B, 11B2, 12A, 12B1, 12B2, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23, 24, 25, 26, 27, 3A1A1A1, 3A1A2, 3A1B1, 3A1B2, 3A2, 3A3, 3B1, 3B1A2, 3B1B, 3B2, 3B3, 4A1A, 4A1B, 4A2, 4B, 5, 6, 7, 8, 9A1A, 9A1A1B, 9A1B, 9A2, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -2160,6 +2210,11 @@
           <t>232</t>
         </is>
       </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -2167,6 +2222,11 @@
           <t>233</t>
         </is>
       </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -2174,6 +2234,11 @@
           <t>234</t>
         </is>
       </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>10A, 10B, 10C, 11, 12, 13A1A, 13B, 14A, 14B, 15, 15A2, 16, 17, 18, 19, 1A1A1A1, 1A1A2, 1A2, 1A3, 1B, 1C, 20, 21, 22, 23, 24, 25A, 25B, 26, 27, 28, 29, 2B, 3, 30, 31, 32, 33, 34, 35, 36, 37, 38, 39, 4, 40, 41, 42, 43, 44, 45, 46, 47, 48, 49, 5, 50, 51, 52, 53, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -2181,6 +2246,11 @@
           <t>235</t>
         </is>
       </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>10, 11, 12A1, 12A2, 12A3, 12B, 13, 14, 15, 16, 17, 18, 19, 1A, 1B, 20, 21, 22, 23, 2A1A1A1, 2A1B1, 2A1B2, 2A2A, 2A2B, 2A3A, 2A3B, 2B, 3B, 4A1, 4A2, 4B1, 4B2, 5A1A, 5A1B, 5A2, 5B, 5C, 5D, 6A1A1A1, 6A2, 6B, 6C, 7, 8A1, 8A2, 8B1, 8B2, 9</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -2188,6 +2258,11 @@
           <t>236</t>
         </is>
       </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -2195,6 +2270,11 @@
           <t>237</t>
         </is>
       </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>10A1, 10A2, 10A3, 10A4, 10B, 11, 12A, 12B, 13, 14, 1A1A, 1A1B1, 1A1B2, 1A2A1, 1A2A2, 1A2A3, 1A2B, 1A3A1, 1A3A2, 1A3B1, 1A3B2, 1A3C1, 1A3C2, 1B1, 1B2, 1B3, 1C1A, 1C1B, 1C2, 1D1, 1D2A, 1D2B, 1E, 2, 3A, 3B, 4A, 4B, 5, 6A1A1A, 6A1B, 6A2, 6B, 7A, 7B, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -2202,6 +2282,11 @@
           <t>238</t>
         </is>
       </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2, 3, 4, 5, 6, 7A, 7B, 8B, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -2209,6 +2294,11 @@
           <t>239</t>
         </is>
       </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>07, 08, 09, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 1A1A, 1A2, 1B1A2, 1B1A3, 1B1B1A1A1, 1B2, 1B3, 1C, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 2A1A1A1, 2B, 2C, 2D, 2E, 30, 31, 32, 33, 34, 35, 36, 37, 38, 39, 3A1A1, 3A2, 3A3, 3B, 4, 40, 41, 42, 43, 44, 45, 46, 47, 48, 49, 5, 50, 51, 52, 53, 54, 55, 56, 57, 58, 59, 6, 60, 61, 62, 63, 64, 65, 66, 67, 68, 69, 70, 71, 72, 73</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -2216,6 +2306,11 @@
           <t>24</t>
         </is>
       </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>1, 10, 11A1A, 11A1B, 11A2, 11B, 12A, 12B, 13, 14, 15, 2, 3A, 3B, 4A, 4B, 4C, 5, 6, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -2223,6 +2318,11 @@
           <t>240</t>
         </is>
       </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>1, 10B, 11B1, 11B2, 12A1, 12B, 12C, 12D, 12E, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 2A, 2B1A, 2B1B, 2B2A1, 2B2B, 30, 31, 32, 33, 34, 35, 36, 37, 38, 39, 3A1A1, 3A2, 3B, 40, 41, 42, 4A1A1A, 4A1B, 4A2, 4A3, 4B, 5A1, 5A2, 5B, 5C1A, 5C1B, 5C2, 6, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -2230,6 +2330,11 @@
           <t>241</t>
         </is>
       </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -2237,6 +2342,11 @@
           <t>242</t>
         </is>
       </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -2244,6 +2354,11 @@
           <t>243</t>
         </is>
       </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14A, 14B, 15, 16, 17, 18, 19, 1A, 1B, 2A, 2B, 3A1, 3A2, 3B, 4A, 4B, 5, 6A, 6B, 6C, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -2251,6 +2366,11 @@
           <t>244</t>
         </is>
       </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 2, 3, 4, 5, 6, 7A, 7B1, 7B2, 7B3, 7B4, 7B5, 7C, 7D10, 7D11, 7D1A1A1, 7D2, 7D3, 7D4, 7D5, 7D6, 7D7, 7D8, 7D9, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -2258,6 +2378,11 @@
           <t>245</t>
         </is>
       </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -2265,6 +2390,11 @@
           <t>246</t>
         </is>
       </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -2272,6 +2402,11 @@
           <t>247</t>
         </is>
       </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -2279,6 +2414,11 @@
           <t>248</t>
         </is>
       </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -2286,6 +2426,11 @@
           <t>249</t>
         </is>
       </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>1, 2, 3B1A, 3B1B, 3B2, 4A1, 4A2, 4A3, 5A, 6, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -2293,6 +2438,11 @@
           <t>25</t>
         </is>
       </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 12A, 12B, 13, 2A, 2B, 2C, 3A, 3B, 3C1, 3C2, 3D, 3E, 3F, 4, 5A, 5B1, 5B2, 6A, 6B1, 6B2A, 6B2B, 6B2C, 6B2D, 7, 8A, 8B, 8C, 8D, 9A, 9B, 9C, 9D</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -2300,6 +2450,11 @@
           <t>250</t>
         </is>
       </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2A, 1B2B, 2, 3A1, 3A2, 3B1A, 3B1B, 3B2, 3C, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -2307,6 +2462,11 @@
           <t>251</t>
         </is>
       </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2B1, 2B2, 3, 4B, 5B, 6B, 7</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -2314,6 +2474,11 @@
           <t>252</t>
         </is>
       </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4A, 4B, 4C, 4D, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -2321,6 +2486,11 @@
           <t>253</t>
         </is>
       </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>1, 4B, 5A, 5B, 6B, 7, 8B</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -2328,6 +2498,11 @@
           <t>254</t>
         </is>
       </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 2, 3, 4A, 4B, 5, 6, 7A, 7B, 7C, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -2335,6 +2510,11 @@
           <t>26</t>
         </is>
       </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 10C, 10D, 10E, 10F, 2A, 2B, 3, 4, 5, 6A1A, 6A2, 6A3, 6A4, 6A5, 6A6, 6B, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -2342,6 +2522,11 @@
           <t>27</t>
         </is>
       </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -2349,6 +2534,11 @@
           <t>28</t>
         </is>
       </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D, 3A1, 3A2, 3B, 3C</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -2356,6 +2546,11 @@
           <t>29</t>
         </is>
       </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4, 5A, 5B, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -2363,6 +2558,11 @@
           <t>3</t>
         </is>
       </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6A, 6B, 6C, 6D, 6E, 6F, 6G, 6H, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -2370,6 +2570,11 @@
           <t>30</t>
         </is>
       </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -2377,6 +2582,11 @@
           <t>31</t>
         </is>
       </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -2384,6 +2594,11 @@
           <t>32</t>
         </is>
       </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -2391,6 +2606,11 @@
           <t>33</t>
         </is>
       </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D, 3</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -2398,6 +2618,11 @@
           <t>34</t>
         </is>
       </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 2, 3, 4, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -2405,6 +2630,11 @@
           <t>35</t>
         </is>
       </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5A, 5B, 5C, 5D</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -2412,6 +2642,11 @@
           <t>36</t>
         </is>
       </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4A, 4B, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -2419,6 +2654,11 @@
           <t>37</t>
         </is>
       </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -2426,6 +2666,11 @@
           <t>38</t>
         </is>
       </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -2433,6 +2678,11 @@
           <t>39</t>
         </is>
       </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A1A, 5A1B, 5A2, 5A3, 5B1, 5B2, 5B3, 6, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -2440,6 +2690,11 @@
           <t>4</t>
         </is>
       </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -2447,6 +2702,11 @@
           <t>40</t>
         </is>
       </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2A, 2B, 2C1, 2C2, 2C3, 3, 4A, 4B, 4C, 4D, 4E, 4F, 5</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -2454,6 +2714,11 @@
           <t>41</t>
         </is>
       </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 1A, 1B, 2, 3, 4, 5A, 5B, 5C, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -2461,6 +2726,11 @@
           <t>42</t>
         </is>
       </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A, 12B1, 12B2, 13, 14, 15A, 15B, 15C, 15D, 2, 3, 4, 5, 6, 7, 8A, 8B, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -2468,6 +2738,11 @@
           <t>43</t>
         </is>
       </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -2475,6 +2750,11 @@
           <t>44</t>
         </is>
       </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>1, 10A1, 10A2, 10B, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 3, 4, 5, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -2482,6 +2762,11 @@
           <t>45</t>
         </is>
       </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 3, 4A1, 4A2, 4B, 4C, 4D</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -2489,6 +2774,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4A, 4B, 4C, 5, 6, 7A1, 7A2, 7B</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -2496,6 +2786,11 @@
           <t>47</t>
         </is>
       </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16A, 16B, 2, 3, 4A, 4B, 4C, 4D, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -2503,6 +2798,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A, 12B, 2A, 2B, 2C, 3, 4A, 4B1, 4B2, 4C, 4D1, 4D2, 4E1, 4E2, 4F, 5, 6, 7A, 7B, 8A, 8B, 8C, 8D, 9</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -2510,6 +2810,11 @@
           <t>49</t>
         </is>
       </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B1A, 2B1B, 2B2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -2517,6 +2822,11 @@
           <t>5</t>
         </is>
       </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -2524,6 +2834,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 2A1, 2A2, 2B, 3A, 3B, 3C, 4</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -2531,6 +2846,11 @@
           <t>51</t>
         </is>
       </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 2, 3, 4, 5, 6A1, 6A2, 6B, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -2538,6 +2858,11 @@
           <t>52</t>
         </is>
       </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B1, 3B2, 3B3, 4, 5A1A, 5A1B, 5A2A, 5A2B, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -2545,6 +2870,11 @@
           <t>53</t>
         </is>
       </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D, 3A1, 3A2, 3B, 4, 5A, 5B, 5C1, 5C2</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -2552,6 +2882,11 @@
           <t>54</t>
         </is>
       </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B1A, 3B1B, 3B2</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -2559,6 +2894,11 @@
           <t>55</t>
         </is>
       </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -2566,6 +2906,11 @@
           <t>56</t>
         </is>
       </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -2573,6 +2918,11 @@
           <t>57</t>
         </is>
       </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -2580,6 +2930,11 @@
           <t>58</t>
         </is>
       </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A, 3B, 3C, 3D</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -2587,6 +2942,11 @@
           <t>59</t>
         </is>
       </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -2594,6 +2954,11 @@
           <t>6</t>
         </is>
       </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A, 12B, 2, 3, 4, 5, 6, 7, 8, 9A, 9B, 9C, 9D, 9E, 9F, 9G</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -2601,6 +2966,11 @@
           <t>60</t>
         </is>
       </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B, 2C, 2D, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -2608,11 +2978,21 @@
           <t>61</t>
         </is>
       </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D, 2E</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
           <t>62</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 1G, 3B1, 3B2, 3B3, 3B4, 5, 6A, 6C, 6D, 7A1, 7A2, 7B, 7C, 7D</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 62 village workbooks (sivaramans-llin 2026-10-10T15:50:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Panpakkam_13.376354_80.132208.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Panpakkam_13.376354_80.132208.xlsx
@@ -3002,6 +3002,11 @@
           <t>63</t>
         </is>
       </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -3009,6 +3014,11 @@
           <t>64</t>
         </is>
       </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 1A1, 1A10, 1A11, 1A12, 1A13, 1A14, 1A15, 1A16, 1A17, 1A18, 1A19, 1A2, 1A20, 1A21, 1A22, 1A23, 1A24, 1A25, 1A26, 1A27, 1A28, 1A29, 1A3, 1A30, 1A31, 1A32, 1A33, 1A34, 1A35, 1A36, 1A37, 1A38, 1A39, 1A4, 1A40, 1A41, 1A42, 1A43, 1A44, 1A45, 1A46, 1A47, 1A5, 1A6, 1A7, 1A8, 1A9, 1B1A, 1B1B, 1B2, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 2A1, 2A1B, 2A1C, 2A1D, 2A2, 2B, 2C, 3, 30, 31, 32, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -3016,6 +3026,11 @@
           <t>65</t>
         </is>
       </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -3023,6 +3038,11 @@
           <t>66</t>
         </is>
       </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -3030,6 +3050,11 @@
           <t>67</t>
         </is>
       </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 1A1A, 1A2, 2, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 3, 30, 31, 32, 33, 34, 35, 36, 37, 38, 39, 40, 41, 42, 43, 44, 45, 46, 47, 48, 49, 4A, 4B, 5, 50, 51, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -3037,6 +3062,11 @@
           <t>68</t>
         </is>
       </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>10, 11A, 11B, 12, 13, 14, 15, 16, 17, 18, 19, 1A1A, 1A2, 1B, 1B2, 1C, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 3, 31, 32, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -3044,6 +3074,11 @@
           <t>69</t>
         </is>
       </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 1A1A, 1A2, 1B1, 1B2, 20, 21, 22, 23, 2A, 3A, 3B, 3C, 3D, 4, 5A, 5B1A, 5B2, 6A1A1, 6A2, 6B, 7A1A, 7A2, 7B, 8A, 8B, 8C, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -3051,6 +3086,11 @@
           <t>7</t>
         </is>
       </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -3058,6 +3098,11 @@
           <t>70</t>
         </is>
       </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 1A1A, 1A2, 1B2, 20, 21, 22, 23, 24, 2A2, 2A3, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -3065,6 +3110,11 @@
           <t>71</t>
         </is>
       </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -3072,6 +3122,11 @@
           <t>72</t>
         </is>
       </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 1A, 1B, 1C, 1D, 1E, 1F, 1G, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 30, 3A1A1A, 3A1A1B, 3A1A1C, 3A1A2, 3A1B, 3A2, 3B, 4A1, 4A1B, 4A2, 4A3, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -3079,6 +3134,11 @@
           <t>73</t>
         </is>
       </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -3086,6 +3146,11 @@
           <t>74</t>
         </is>
       </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -3093,6 +3158,11 @@
           <t>75</t>
         </is>
       </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 2A1A, 2A2, 3, 30, 4, 6, 7A1A, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -3100,6 +3170,11 @@
           <t>76</t>
         </is>
       </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>10, 1A1A, 1B, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -3107,6 +3182,11 @@
           <t>77</t>
         </is>
       </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 1A1, 1B, 1C, 1D, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -3114,6 +3194,11 @@
           <t>78</t>
         </is>
       </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 1A1A1, 1B, 1C, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -3121,6 +3206,11 @@
           <t>79</t>
         </is>
       </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>10, 12, 13, 14, 15, 16, 17, 1A1, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -3128,6 +3218,11 @@
           <t>8</t>
         </is>
       </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A, 12B, 2, 3A, 3B, 4, 5, 6A1, 6A2, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -3135,6 +3230,11 @@
           <t>80</t>
         </is>
       </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 1A1A, 2, 20, 21, 22, 23, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -3142,6 +3242,11 @@
           <t>81</t>
         </is>
       </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>1A1A1, 1B, 2, 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -3149,6 +3254,11 @@
           <t>82</t>
         </is>
       </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 1A1A, 1A2, 1A3, 1B, 1C, 20, 21, 22, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -3156,6 +3266,11 @@
           <t>83</t>
         </is>
       </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -3163,6 +3278,11 @@
           <t>84</t>
         </is>
       </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -3170,6 +3290,11 @@
           <t>85</t>
         </is>
       </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -3177,6 +3302,11 @@
           <t>86</t>
         </is>
       </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -3184,6 +3314,11 @@
           <t>87</t>
         </is>
       </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -3191,6 +3326,11 @@
           <t>88</t>
         </is>
       </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>1, 2A1A1A1, 2A1A1A2, 2A1A1B, 2A1B, 2A2, 2B, 2C, 2D</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -3198,6 +3338,11 @@
           <t>89</t>
         </is>
       </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2, 3A, 3B, 4A, 4B, 5</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -3205,6 +3350,11 @@
           <t>9</t>
         </is>
       </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4A, 4B1, 4B2, 5A, 5B, 6A, 6B, 6C, 6D</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -3212,6 +3362,11 @@
           <t>90</t>
         </is>
       </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -3219,6 +3374,11 @@
           <t>91</t>
         </is>
       </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -3226,6 +3386,11 @@
           <t>92</t>
         </is>
       </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2A1, 2B, 3A1A1A, 3A1B, 3A2, 3B, 4A1A, 4A2, 4B, 4C, 4D1, 4D2, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -3233,6 +3398,11 @@
           <t>93</t>
         </is>
       </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>10A, 10B, 11, 12A, 12B, 13, 14A, 14B, 15A, 15B, 16A, 16B, 17A1, 17A2, 17B, 18, 19A, 19B, 1A, 1B, 20A, 20B, 2A1A, 2A1B, 2A2A, 2A2B1, 2A2B2, 2A2B3, 2B1, 2B2A1, 2B2A2, 2B2B, 2C1A, 2C1B, 2C2, 3, 4A1, 4A2, 4B, 5A1, 5A2, 5B, 6A, 6B, 7A1, 7A2, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -3240,6 +3410,11 @@
           <t>94</t>
         </is>
       </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>10A1, 10A2, 10B, 11A1, 11A2, 11B, 12, 13, 14, 15A1, 15A2, 15B, 16A1, 16A2, 16B, 17, 18, 19, 1A, 1B, 2, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 3, 30, 31, 32, 33, 34, 4, 5, 6A1A, 6A2, 6A3, 6A4, 6A5, 6B, 7, 8A1A, 8A2A, 8A2B, 8B, 9A, 9B, 9C, 9D</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -3247,6 +3422,11 @@
           <t>95</t>
         </is>
       </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14A, 14B, 15A1, 15A2, 15B, 16A1A, 16A1B, 16A2A, 16A2B, 16A3A, 16A3B, 16B, 2A, 2B, 3A1A, 3A1B, 3A2, 4B1, 4B2, 5B, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -3254,6 +3434,11 @@
           <t>96</t>
         </is>
       </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13A1, 13A2, 13B, 14A1, 14A2, 14B, 15A1A, 15A1B, 15A2, 15B, 2, 3A1, 3A2, 3B, 4A1, 4A2, 4B, 5A1, 5A2, 5B, 6A1, 6A2, 6B, 7A1A1, 7A1A2, 7A1B, 7A2A, 7A2B, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -3261,6 +3446,11 @@
           <t>97</t>
         </is>
       </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -3268,11 +3458,21 @@
           <t>98</t>
         </is>
       </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
           <t>99</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>